<commit_message>
Implement email tracking and dashboard features
</commit_message>
<xml_diff>
--- a/data/sent.xlsx
+++ b/data/sent.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D47"/>
+  <dimension ref="A1:D64"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1060,9 +1060,247 @@
         <v/>
       </c>
     </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>gavaliashutosh490@gmail.com</v>
+      </c>
+      <c r="B48" t="str">
+        <v>Murphy Mombo</v>
+      </c>
+      <c r="C48" t="str">
+        <v>Application for MERN Stack Developer Role — Immediate Joiner | 3 Yrs Experience</v>
+      </c>
+      <c r="D48" t="str">
+        <v>Cannot read properties of undefined (reading 'host')</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <v>gavaliashutosh490@gmail.com</v>
+      </c>
+      <c r="B49" t="str">
+        <v>Murphy Mombo</v>
+      </c>
+      <c r="C49" t="str">
+        <v>Application for MERN Stack Developer Role — Immediate Joiner | 3 Yrs Experience</v>
+      </c>
+      <c r="D49" t="str">
+        <v>Cannot read properties of undefined (reading 'host')</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="str">
+        <v>gavaliashutosh490@gmail.com</v>
+      </c>
+      <c r="B50" t="str">
+        <v>Murphy Mombo</v>
+      </c>
+      <c r="C50" t="str">
+        <v>Application for MERN Stack Developer Role — Immediate Joiner | 3 Yrs Experience</v>
+      </c>
+      <c r="D50" t="str">
+        <v>Cannot read properties of undefined (reading 'host')</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="str">
+        <v>gavaliashutosh490@gmail.com</v>
+      </c>
+      <c r="B51" t="str">
+        <v>Murphy Mombo</v>
+      </c>
+      <c r="C51" t="str">
+        <v>Application for MERN Stack Developer Role — Immediate Joiner | 3 Yrs Experience</v>
+      </c>
+      <c r="D51" t="str">
+        <v>Cannot read properties of undefined (reading 'host')</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="str">
+        <v>gavaliashutosh490@gmail.com</v>
+      </c>
+      <c r="B52" t="str">
+        <v>Murphy Mombo</v>
+      </c>
+      <c r="C52" t="str">
+        <v>Application for MERN Stack Developer Role — Immediate Joiner | 3 Yrs Experience</v>
+      </c>
+      <c r="D52" t="str">
+        <v>Cannot read properties of undefined (reading 'host')</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="str">
+        <v>gavaliashutosh490@gmail.com</v>
+      </c>
+      <c r="B53" t="str">
+        <v>he</v>
+      </c>
+      <c r="C53" t="str">
+        <v>Application for MERN Stack Developer Role — Immediate Joiner | 3 Yrs Experience</v>
+      </c>
+      <c r="D53" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="str">
+        <v>mombomurphy219@gmail.com</v>
+      </c>
+      <c r="B54" t="str">
+        <v>Murphy Mombo</v>
+      </c>
+      <c r="C54" t="str">
+        <v>Application for MERN Stack Developer Role — Immediate Joiner | 3 Yrs Experience</v>
+      </c>
+      <c r="D54" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="str">
+        <v>bhavya@jpstechsolutions.com</v>
+      </c>
+      <c r="B55" t="str">
+        <v/>
+      </c>
+      <c r="C55" t="str">
+        <v>Application for React Native Developer Role — Immediate Joiner | 3 Yrs Experience</v>
+      </c>
+      <c r="D55" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="str">
+        <v>mike@intellisofttech.com</v>
+      </c>
+      <c r="B56" t="str">
+        <v/>
+      </c>
+      <c r="C56" t="str">
+        <v>Application for React Native Developer Role — Immediate Joiner | 3 Yrs Experience</v>
+      </c>
+      <c r="D56" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="str">
+        <v>tehseen@versanteconsulting.com</v>
+      </c>
+      <c r="B57" t="str">
+        <v/>
+      </c>
+      <c r="C57" t="str">
+        <v>Application for React Native Developer Role — Immediate Joiner | 3 Yrs Experience</v>
+      </c>
+      <c r="D57" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="str">
+        <v>priyanka.choudhari@citi.com</v>
+      </c>
+      <c r="B58" t="str">
+        <v/>
+      </c>
+      <c r="C58" t="str">
+        <v>Application for React Native Developer Role — Immediate Joiner | 3 Yrs Experience</v>
+      </c>
+      <c r="D58" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="str">
+        <v>mrilo5555@gmail.com</v>
+      </c>
+      <c r="B59" t="str">
+        <v>hy</v>
+      </c>
+      <c r="C59" t="str">
+        <v>Application for MERN Stack Developer Role — Immediate Joiner | 3 Yrs Experience</v>
+      </c>
+      <c r="D59" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="str">
+        <v>ashutosh38agg38@gmail.com</v>
+      </c>
+      <c r="B60" t="str">
+        <v>hr</v>
+      </c>
+      <c r="C60" t="str">
+        <v>Application for MERN Stack Developer Role — Immediate Joiner | 3 Yrs Experience</v>
+      </c>
+      <c r="D60" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="str">
+        <v>ashutosh38agg38@gmail.com</v>
+      </c>
+      <c r="B61" t="str">
+        <v>hr</v>
+      </c>
+      <c r="C61" t="str">
+        <v>Application for MERN Stack Developer Role — Immediate Joiner | 3 Yrs Experience</v>
+      </c>
+      <c r="D61" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="str">
+        <v>ashutosh38agg38@gmail.com</v>
+      </c>
+      <c r="B62" t="str">
+        <v>hr</v>
+      </c>
+      <c r="C62" t="str">
+        <v>Application for MERN Stack Developer Role — Immediate Joiner | 3 Yrs Experience</v>
+      </c>
+      <c r="D62" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="str">
+        <v>ashutosh38agg38@gmail.com</v>
+      </c>
+      <c r="B63" t="str">
+        <v>hr</v>
+      </c>
+      <c r="C63" t="str">
+        <v>Application for MERN Stack Developer Role — Immediate Joiner | 3 Yrs Experience</v>
+      </c>
+      <c r="D63" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="str">
+        <v>ashutosh38agg38@gmail.com</v>
+      </c>
+      <c r="B64" t="str">
+        <v>he</v>
+      </c>
+      <c r="C64" t="str">
+        <v>Application for MERN Stack Developer Role — Immediate Joiner | 3 Yrs Experience</v>
+      </c>
+      <c r="D64" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D47"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D64"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add HR Finder Job Board Email Extractor with live SSE streaming, parallel extraction, Render keepalive and concurrency fixes
</commit_message>
<xml_diff>
--- a/data/sent.xlsx
+++ b/data/sent.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D64"/>
+  <dimension ref="A1:D87"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1298,9 +1298,334 @@
         <v/>
       </c>
     </row>
+    <row r="65">
+      <c r="A65" t="str">
+        <v>hr@company.com</v>
+      </c>
+      <c r="B65" t="str">
+        <v>Hiring Team</v>
+      </c>
+      <c r="C65" t="str">
+        <v>Application for MERN Stack Developer Role — Immediate Joiner | 3 Yrs Experience</v>
+      </c>
+      <c r="D65" t="str">
+        <v>ENOENT: no such file or directory, open 'F:\JobReach-main\JobReach-main\data\default-resume.pdf'</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="str">
+        <v>recruiter@company.com</v>
+      </c>
+      <c r="B66" t="str">
+        <v>Priya</v>
+      </c>
+      <c r="C66" t="str">
+        <v>Application for MERN Stack Developer Role — Immediate Joiner | 3 Yrs Experience</v>
+      </c>
+      <c r="D66" t="str">
+        <v>ENOENT: no such file or directory, open 'F:\JobReach-main\JobReach-main\data\default-resume.pdf'</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="str">
+        <v>hr@company.com</v>
+      </c>
+      <c r="B67" t="str">
+        <v>Hiring Team</v>
+      </c>
+      <c r="C67" t="str">
+        <v>Application for MERN Stack Developer Role — Immediate Joiner | 3 Yrs Experience</v>
+      </c>
+      <c r="D67" t="str">
+        <v>ENOENT: no such file or directory, open 'F:\JobReach-main\JobReach-main\data\default-resume.pdf'</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="str">
+        <v>recruiter@company.com</v>
+      </c>
+      <c r="B68" t="str">
+        <v>Priya</v>
+      </c>
+      <c r="C68" t="str">
+        <v>Application for MERN Stack Developer Role — Immediate Joiner | 3 Yrs Experience</v>
+      </c>
+      <c r="D68" t="str">
+        <v>ENOENT: no such file or directory, open 'F:\JobReach-main\JobReach-main\data\default-resume.pdf'</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="str">
+        <v>hr@company.com</v>
+      </c>
+      <c r="B69" t="str">
+        <v>Hiring Team</v>
+      </c>
+      <c r="C69" t="str">
+        <v>Application for MERN Stack Developer Role — Immediate Joiner | 3 Yrs Experience</v>
+      </c>
+      <c r="D69" t="str">
+        <v>ENOENT: no such file or directory, open 'F:\JobReach-main\JobReach-main\data\default-resume.pdf'</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="str">
+        <v>recruiter@company.com</v>
+      </c>
+      <c r="B70" t="str">
+        <v>Priya</v>
+      </c>
+      <c r="C70" t="str">
+        <v>Application for MERN Stack Developer Role — Immediate Joiner | 3 Yrs Experience</v>
+      </c>
+      <c r="D70" t="str">
+        <v>ENOENT: no such file or directory, open 'F:\JobReach-main\JobReach-main\data\default-resume.pdf'</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="str">
+        <v>yoginiphalak513@gmail.com</v>
+      </c>
+      <c r="B71" t="str">
+        <v/>
+      </c>
+      <c r="C71" t="str">
+        <v>Application for MERN Stack Developer Role — Immediate Joiner | 3 Yrs Experience</v>
+      </c>
+      <c r="D71" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="str">
+        <v>pawarshubham1295@gmail.com</v>
+      </c>
+      <c r="B72" t="str">
+        <v/>
+      </c>
+      <c r="C72" t="str">
+        <v>Application for MERN Stack Developer Role — Immediate Joiner | 3 Yrs Experience</v>
+      </c>
+      <c r="D72" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="str">
+        <v>yoginiphalak513@gmail.com</v>
+      </c>
+      <c r="B73" t="str">
+        <v/>
+      </c>
+      <c r="C73" t="str">
+        <v>Application for MERN Stack Developer Role — Immediate Joiner | 3 Yrs Experience</v>
+      </c>
+      <c r="D73" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="str">
+        <v>pawarshubham1295@gmail.com</v>
+      </c>
+      <c r="B74" t="str">
+        <v/>
+      </c>
+      <c r="C74" t="str">
+        <v>Application for MERN Stack Developer Role — Immediate Joiner | 3 Yrs Experience</v>
+      </c>
+      <c r="D74" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="str">
+        <v>yoginiphalak513@gmail.com</v>
+      </c>
+      <c r="B75" t="str">
+        <v/>
+      </c>
+      <c r="C75" t="str">
+        <v>Application for MERN Stack Developer Role — Immediate Joiner | 3 Yrs Experience</v>
+      </c>
+      <c r="D75" t="str">
+        <v>Invalid login: 535 5.7.8 Authentication failed</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="str">
+        <v>pawarshubham1295@gmail.com</v>
+      </c>
+      <c r="B76" t="str">
+        <v/>
+      </c>
+      <c r="C76" t="str">
+        <v>Application for MERN Stack Developer Role — Immediate Joiner | 3 Yrs Experience</v>
+      </c>
+      <c r="D76" t="str">
+        <v>Invalid login: 535 5.7.8 Authentication failed</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="str">
+        <v>ashuagd@gmail.com</v>
+      </c>
+      <c r="B77" t="str">
+        <v/>
+      </c>
+      <c r="C77" t="str">
+        <v>Application for MERN Stack Developer Role — Immediate Joiner | 3 Yrs Experience</v>
+      </c>
+      <c r="D77" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="str">
+        <v>ashutosh38agg38@gmail.com</v>
+      </c>
+      <c r="B78" t="str">
+        <v/>
+      </c>
+      <c r="C78" t="str">
+        <v>Application for MERN Stack Developer Role — Immediate Joiner | 3 Yrs Experience</v>
+      </c>
+      <c r="D78" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="str">
+        <v>ashuagd@gmail.com</v>
+      </c>
+      <c r="B79" t="str">
+        <v/>
+      </c>
+      <c r="C79" t="str">
+        <v>Application for MERN Stack Developer Role — Immediate Joiner | 3 Yrs Experience</v>
+      </c>
+      <c r="D79" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="str">
+        <v>ashutosh38agg38@gmail.com</v>
+      </c>
+      <c r="B80" t="str">
+        <v/>
+      </c>
+      <c r="C80" t="str">
+        <v>Application for MERN Stack Developer Role — Immediate Joiner | 3 Yrs Experience</v>
+      </c>
+      <c r="D80" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="str">
+        <v>ashutosh38agg38@gmail.com</v>
+      </c>
+      <c r="B81" t="str">
+        <v/>
+      </c>
+      <c r="C81" t="str">
+        <v>Application for MERN Stack Developer Role — Immediate Joiner | 3 Yrs Experience</v>
+      </c>
+      <c r="D81" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="str">
+        <v>ashutosh38agg38@gmail.com</v>
+      </c>
+      <c r="B82" t="str">
+        <v/>
+      </c>
+      <c r="C82" t="str">
+        <v>Application for MERN Stack Developer Role — Immediate Joiner | 3 Yrs Experience</v>
+      </c>
+      <c r="D82" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="str">
+        <v>ashutosh38agg38@gmail.com</v>
+      </c>
+      <c r="B83" t="str">
+        <v/>
+      </c>
+      <c r="C83" t="str">
+        <v>Application for MERN Stack Developer Role — Immediate Joiner | 3 Yrs Experience</v>
+      </c>
+      <c r="D83" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="84" xml:space="preserve">
+      <c r="A84" t="str">
+        <v>ashutosh38agg38@gmail.com</v>
+      </c>
+      <c r="B84" t="str">
+        <v/>
+      </c>
+      <c r="C84" t="str">
+        <v>Application for React Developer Role — Immediate Joiner | 3 Yrs Experience</v>
+      </c>
+      <c r="D84" t="str" xml:space="preserve">
+        <v xml:space="preserve">Invalid login: 535-5.7.8 Username and Password not accepted. For more information, go to
+535 5.7.8  https://support.google.com/mail/?p=BadCredentials d2e1a72fcca58-8296c9f83f3sm2067731b3a.0 - gsmtp</v>
+      </c>
+    </row>
+    <row r="85" xml:space="preserve">
+      <c r="A85" t="str">
+        <v>ashutosh38agg38@gmail.com</v>
+      </c>
+      <c r="B85" t="str">
+        <v/>
+      </c>
+      <c r="C85" t="str">
+        <v>Application for React Developer Role — Immediate Joiner | 3 Yrs Experience</v>
+      </c>
+      <c r="D85" t="str" xml:space="preserve">
+        <v xml:space="preserve">Invalid login: 535-5.7.8 Username and Password not accepted. For more information, go to
+535 5.7.8  https://support.google.com/mail/?p=BadCredentials d2e1a72fcca58-82739d4d826sm18779695b3a.10 - gsmtp</v>
+      </c>
+    </row>
+    <row r="86" xml:space="preserve">
+      <c r="A86" t="str">
+        <v>ashuagd@gmail.com</v>
+      </c>
+      <c r="B86" t="str">
+        <v/>
+      </c>
+      <c r="C86" t="str">
+        <v>Application for React Developer Role — Immediate Joiner | 3 Yrs Experience</v>
+      </c>
+      <c r="D86" t="str" xml:space="preserve">
+        <v xml:space="preserve">Invalid login: 535-5.7.8 Username and Password not accepted. For more information, go to
+535 5.7.8  https://support.google.com/mail/?p=BadCredentials d2e1a72fcca58-8296c9f83f3sm2071165b3a.0 - gsmtp</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="str">
+        <v>ashuagd@gmail.com</v>
+      </c>
+      <c r="B87" t="str">
+        <v/>
+      </c>
+      <c r="C87" t="str">
+        <v>Application for React Developer Role — Immediate Joiner | 3 Yrs Experience</v>
+      </c>
+      <c r="D87" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D64"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D87"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>